<commit_message>
Mitarbeiter-Kalender: offene Frage geklärt (nur eigene Termine)
Nutzer-Klarstellung eingearbeitet: der Monteur sieht nur seine eigenen
Termine. Zuweisung erfolgt pro datiertem Termin (appointment_employees);
der Termin gehoert zu einem Projekt und erscheint mit dessen Infos.
"Projekt zugewiesen" und "nur eigene" sind dasselbe Modell.

Angezeigte Felder frei definierbar (SELECT/Join), Feldliste vor
Umsetzung. Sicherheitshinweis praezisiert: MS-Login gilt nur im Browser,
an die Middleware geht ein statisches VITE_API_TOKEN (apiClient.ts:47/188)
- "nur eigene" ist unter Variante A Anzeige-Logik, erzwungen erst mit B.

Nur Text (Belege/Backlog), keine Zahlenaenderung: Terminplanung bleibt
53-86 h.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/aufwandsschaetzung-4-topics.xlsx
+++ b/aufwandsschaetzung-4-topics.xlsx
@@ -2379,7 +2379,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G47"/>
+  <dimension ref="B2:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -3165,26 +3165,33 @@
     <row r="44">
       <c r="B44" s="42" t="inlineStr">
         <is>
-          <t>· OFFENE FRAGE Phase 3: Zeigt der Mitarbeiter-Kalender nur Termine, denen er per appointment_employees zugewiesen ist, ODER alle Termine der Projekte, denen er zugewiesen ist? Ersteres ist sauberer und angenommen; Letzteres bräuchte zusätzlich die (ggf. fuzzy/datumslose) Projekt-Ebene. Klären.</t>
+          <t>· GEKLÄRT 2026-07-27: Monteur sieht NUR seine eigenen Termine. Der BO weist ihn einem datierten Termin zu (appointment_employees); dieser Termin gehört zu Projekt A und erscheint mit dessen Infos. „Projekt zugewiesen → erscheint" und „nur eigene" sind dasselbe Modell.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="42" t="inlineStr">
         <is>
-          <t>· Sicherheitshinweis Phase 3: Unter Variante A (Shared Secret) kann technisch jeder Mitarbeiter den Kalender jedes anderen abfragen (id im Request austauschbar). Gleiche Ausgangslage wie im ganzen Tool heute — echte Absicherung erst mit RBAC Variante B.</t>
+          <t>· Sicherheitshinweis Phase 3: MS-Login gilt nur im Browser — an die Middleware geht ein statisches VITE_API_TOKEN (apiClient.ts:47/188), für alle identisch. Unter Variante A ist „nur eigene" reine Anzeige-Logik; jeder könnte die id austauschen. Technisch erzwungen erst mit RBAC Variante B.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="42" t="inlineStr">
         <is>
-          <t>· BESTÄTIGT positiv: WhatsApp läuft über Twilio, produktiv. Die Zuweisungs-Benachrichtigung ist live und eine belastbare Vorlage.</t>
+          <t>· Anzeige frei definierbar: welche DB-Felder ans Kalender-Event kommen (Projekt, Adresse, Datum/ganztägig, Notiz, Status, Link), legen wir per SELECT/Join fest. Vorlage: der bestehende ICS-Export (ConstructionSiteList.vue:462). Feldliste vor Umsetzung vereinbaren.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="42" t="inlineStr">
+        <is>
+          <t>· BESTÄTIGT positiv: WhatsApp läuft über Twilio, produktiv. Die Zuweisungs-Benachrichtigung ist live und eine belastbare Vorlage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="42" t="inlineStr">
         <is>
           <t>· Kundenaussage bleibt gültig und dämpft den Umfang: keine Stundenangaben nötig, „Monteur A ist Montag auf Baustelle XY" reicht.</t>
         </is>

</xml_diff>

<commit_message>
Entscheidung festgehalten: Auth-Variante A, B als Technical Debt
Nutzer-Entscheidung 2026-07-27: RBAC bleibt Anzeige-Logik (Variante A).
Serverseitige Durchsetzung (Variante B) wird bewusst als Technical Debt
aufgeschoben.

Dokumentiert in:
- aufwandsschaetzung-4-topics.xlsx: Dropdown-Hinweis + Technical-Debt-
  Spezifikation in den RBAC-Belegen (was offen bleibt, wann faellig,
  Nachruestkosten +19-30 h).
- ROADMAP-v2.md: Entscheidungsblock im Code-Analyse-Kasten.
- rollen-rechteverwaltung/BACKLOG.md: eigener Technical-Debt-Abschnitt
  mit Umfang von Variante B und Ausloesern zum Abbau.

Konsequenz bis zum Abbau: "nur eigene Daten" und Admin-/Rollen-Sperren
sind Anzeige-Logik, keine serverseitige Sperre. Keine Zahlenaenderung
an der Grundschaetzung.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/aufwandsschaetzung-4-topics.xlsx
+++ b/aufwandsschaetzung-4-topics.xlsx
@@ -725,7 +725,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>← A = RBAC bleibt Anzeige-Logik · B = serverseitig durchgesetzt</t>
+          <t>← ENTSCHIEDEN 2026-07-27: A. B (serverseitig durchgesetzt) als Technical Debt vermerkt.</t>
         </is>
       </c>
     </row>
@@ -1430,7 +1430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G34"/>
+  <dimension ref="B2:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1961,7 +1961,21 @@
     <row r="34">
       <c r="B34" s="42" t="inlineStr">
         <is>
-          <t>· ENTSCHEIDUNG: Variante A schützt vor Verwechslung, nicht vor Absicht. Für ein internes Tool mit 10 Leuten kann das legitim sein — aber bewusst und dem Kunden gegenüber benannt.</t>
+          <t>· ENTSCHEIDUNG 2026-07-27: Variante A. B wird bewusst als Technical Debt aufgeschoben.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="42" t="inlineStr">
+        <is>
+          <t>· TECHNICAL DEBT (offen): Der Server authentifiziert den einzelnen Nutzer NICHT. Folgen: (1) „nur eigene Daten" ist reine Anzeige-Logik; (2) Admin-/Rollen-Sperren sind UI-only, nicht serverseitig erzwungen; (3) das VITE_API_TOKEN ist aus dem Browser-Bundle auslesbar und für alle gleich.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="42" t="inlineStr">
+        <is>
+          <t>· Fällig spätestens wenn: heikle Daten dazukommen, ein nicht vertrauenswürdiger Nutzer Zugang hat, oder eine Rolle (z. B. Zeichner) etwas wirklich NICHT auslösen können darf statt es nur nicht zu sehen. Nachrüstkosten dann = Variante B (+19–30 h, ggf. mehr bei mehr Endpunkten).</t>
         </is>
       </c>
     </row>

</xml_diff>